<commit_message>
Cross-check key figures and correct labels
- How to Fish: anchor on GameDiscoverCo's corroborated August readout
- PEAK cost and RV There Yet? build time marked as reported, single-source
- Remove internal research jargon from data files

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6mDjnjeBZpi9xGXrpYz1n
</commit_message>
<xml_diff>
--- a/game-market-research/games_analysis.xlsx
+++ b/game-market-research/games_analysis.xlsx
@@ -901,7 +901,7 @@
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>core team of ~10 people plus contributors (remote) [CONFIRMED in substance – PCGamesN/GeekWire, per coordinator-verified lead]; an 8-person crew ran the Oct 2023 Godot test jam ('Dancing Duelists') [secondary source case study]</t>
+          <t>core team of ~10 people plus contributors (remote) [CONFIRMED in substance – PCGamesN/GeekWire, re-confirmed in a cross-check search on 2026-10-08]; an 8-person crew ran the Oct 2023 Godot test jam ('Dancing Duelists') [secondary source case study]</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -1149,7 +1149,7 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>&lt; $200,000 total [CONFIRMED – Aggro Crab studio head Nick Kaman, GDC talk via Game Developer]. Cross-check: 7 people × ~1–4 months × $6k ≈ $42k–170k [ESTIMATE].</t>
+          <t>~$200,000 total [ESTIMATE/reported – a single secondary (Italian-language) press report of the developers' figure; the 'under $200k' wording and the GDC 2026 talk ('Putting the Friends in Friendslop', Nick Kaman) could not be confirmed as the source in a cross-check on 2026-10-08]. Cross-check: 7 people × ~1–4 months × $6k ≈ $42k–170k [ESTIMATE].</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>Units: 10M+ (Aug 2025, Keighley/Alinea) and '11M on Steam' (GamesRadar 2026 headline) vs Raijin's ~7M (June 2026), which is clearly an underestimate; used 10–11M. The lead of 15.7M units / $87–92M could not be found in any source and was not used. '20M players' (June 2026, Aggro Crab) counts players, not purchases. Price: list $7.99 but launched at 38% off (~$4.95) and frequently discounted, so used Alinea's implied ~$5.67 realised price instead of 0.75 × list. Dev time: '4 weeks' (core jam) vs '~4 months' (total) – both reported. Peak CCU: 169,910–171k across trackers; used SteamDB-reported 170,759.</t>
+          <t>Units: 10M+ (Aug 2025, Keighley/Alinea) and '11M on Steam' (GamesRadar 2026 headline) vs Raijin's ~7M (June 2026), which is clearly an underestimate; used 10–11M. The lead of 15.7M units / $87–92M could not be found in any source and was not used. '20M players' (June 2026, Aggro Crab) counts players, not purchases. Price: list $7.99 but launched at 38% off (~$4.95) and frequently discounted, so used Alinea's implied ~$5.67 realised price instead of 0.75 × list. Dev time: '4 weeks' (core jam) vs '~4 months' (total) – both reported. Peak CCU: 169,910–171k across trackers; used SteamDB-reported 170,759. CROSS-CHECK 2026-10-08: the production-cost figure was downgraded from CONFIRMED to reported/ESTIMATE because no English-language primary source was found.</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t>~9 weeks: core fixed in 1 week, then ~8 weeks to launch [CONFIRMED – devs via Automaton/GamesIndustry.biz]; CEO: launched 'just eight weeks after development began' [CONFIRMED – Tim Badylak LinkedIn]. Press variously reports '3 months' and 'game-jam project in summer 2025' (Icy Veins, Wikipedia)</t>
+          <t>~2–3 months: core fixed in ~1 week, then ~8 weeks to launch [reported – devs via Automaton/GamesIndustry.biz (Nordic Game 2026) and CEO Tim Badylak on LinkedIn ('launched just eight weeks after development began')]; Wikipedia/Icy Veins describe a summer-2025 game-jam project; press also says '3 months'. A cross-check search on 2026-10-08 could not re-find the interview, so treat '~9 weeks' as reported, not independently verified.</t>
         </is>
       </c>
       <c r="X11" s="3" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="AF11" s="3" t="inlineStr">
         <is>
-          <t>Week-1 sales: 1.3M (dev CM, 2025-10-26/27) vs a report of '2.5M in first week' – the CEO's LinkedIn actually says 2.5M within two weeks; used that. A gamedev.net/GamesIndustry syndication said '2M units in eight days' – consistent with the trajectory. Dev time: '8 weeks' (CEO), '1 week + ~8 weeks' (Automaton), '3 months' (Icy Veins) – used ~9 weeks. Team: 4 devs built it (dev interview) vs 'five-person studio' (review) – 4 used for the game. Steam units now: Raijin 2.1M (contradicts confirmed 4.5M, discarded) vs Gamalytic 7.3M vs Boxleiter 5.3–7.1M – reported a range. Gross: Raijin $14M vs Gamalytic $45.4M vs own $27–36M. Xbox Game Pass date: Pure Xbox metadata May 2026 vs Xbox Wire 2026-06-30 – used Xbox Wire. Exact US price ($7.99 vs $8.99) not verified; GameDiscoverCo and Notebookcheck both say '$8'</t>
+          <t>Week-1 sales: 1.3M (dev CM, 2025-10-26/27) vs a report of '2.5M in first week' – the CEO's LinkedIn actually says 2.5M within two weeks; used that. A gamedev.net/GamesIndustry syndication said '2M units in eight days' – consistent with the trajectory. Dev time: '8 weeks' (CEO), '1 week + ~8 weeks' (Automaton), '3 months' (Icy Veins) – used ~9 weeks. Team: 4 devs built it (dev interview) vs 'five-person studio' (review) – 4 used for the game. Steam units now: Raijin 2.1M (contradicts confirmed 4.5M, discarded) vs Gamalytic 7.3M vs Boxleiter 5.3–7.1M – reported a range. Gross: Raijin $14M vs Gamalytic $45.4M vs own $27–36M. Xbox Game Pass date: Pure Xbox metadata May 2026 vs Xbox Wire 2026-06-30 – used Xbox Wire. Exact US price ($7.99 vs $8.99) not verified; GameDiscoverCo and Notebookcheck both say '$8' CROSS-CHECK 2026-10-08: the 4-developer / ~9-week build could not be re-found in an independent search; the 4.5M-by-December-2025 figure was corroborated by an aggregator (2.5–4.5M range).</t>
         </is>
       </c>
       <c r="AG11" s="3" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="P13" s="3" t="inlineStr">
         <is>
-          <t>1,000,000 copies by 2026-08-22, i.e. ~48 h after launch [CONFIRMED – dev Steam news post '1 MILLION FISHERMEN IN 2 DAYS', via GamesRadar, Sweden Game Arena, Dot Esports]. &gt;6.3M units by end of Aug 2026 [ESTIMATE – GameDiscoverCo Aug-2026 report]. &gt;8.5M units lifetime by end of Sep 2026 [ESTIMATE – GameDiscoverCo Sep-2026 report, Steam only, excludes keys]. Boxleiter cross-check: ~69,000 all-language reviews (late Sep 2026 snapshot) × 80 (implied ratio at the 1M milestone) ≈ 5.5M; × 120 ≈ 8.3M [ESTIMATE]. Steam Page Analyzer's low-multiplier model gives only ~593k (395k–791k), which the confirmed 1M already exceeds, so disregard it. Dev target had been ~200,000 copies [CONFIRMED – Olsson via Sweden Game Arena]. No dev-announced milestone beyond 1M found as of 2026-10-08.</t>
+          <t>1,000,000 copies by 2026-08-22, i.e. ~48 h after launch [CONFIRMED – dev Steam news post '1 MILLION FISHERMEN IN 2 DAYS', via GamesRadar, Sweden Game Arena, Dot Esports]. 6.3M+ units sold in August 2026 alone, the month's #1 new PC/console release by units [ESTIMATE – GameDiscoverCo August-2026 readout, corroborated by two secondary reports (Cinevva, 2026-09-04)]. A later GameDiscoverCo September readout reportedly put lifetime Steam units above 8.5M [ESTIMATE – could NOT be independently re-verified in a 2026-10-08 cross-check; treat as an upper scenario]. Boxleiter cross-check: ~69,000 all-language reviews (late Sep 2026) × 80 (implied ratio at the 1M milestone) ≈ 5.5M [ESTIMATE]. Steam Page Analyzer's ~593k is below the confirmed 1M and is disregarded. The developers had targeted ~200,000 copies [CONFIRMED – Olsson via Sweden Game Arena]. No dev-announced milestone beyond 1M found as of 2026-10-08.</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
@@ -2799,17 +2799,17 @@
       </c>
       <c r="S13" s="3" t="inlineStr">
         <is>
-          <t>~77–83 at the 1M milestone (1,000,000 CONFIRMED units ÷ ~12,000–13,000 reviews on 2026-08-22/23). Use ~80 as the calibration point for cheap viral friendslop. If GameDiscoverCo's &gt;8.5M (end Sep) is right, the ratio vs ~69k reviews is ~120+. That is an estimate on an estimate, but it suggests the ratio grows after the launch spike.</t>
+          <t>~77–83 at the 1M milestone (1,000,000 CONFIRMED units ÷ ~12,000–13,000 reviews on 2026-08-22/23). Use ~80 as the calibration point for cheap viral friendslop. Versus ~61k reviews on 2026-09-12, GameDiscoverCo's 6.3M+ August units imply ≥100× [ESTIMATE].</t>
         </is>
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>&gt;$38M lifetime Steam gross through Sep 2026 [ESTIMATE – GameDiscoverCo Sep-2026 report]. GDCo August chart: ~$26M gross in Aug 2026, #2 new Steam release by revenue [ESTIMATE – GameDiscoverCo]. Spec method cross-check: 8.5M × ($7.99 × 0.75 = $5.99) ≈ $51M. That overstates the total because most units (≥6.3M of 8.5M) sold during the $4.95 launch week or under regional pricing. GDCo's figure implies ~$4.47 per unit, which is consistent with that. Chosen central value ≈ $38M (range $32M–$51M).</t>
+          <t>≈ $26M Steam gross in August 2026 alone [ESTIMATE – GameDiscoverCo August readout, corroborated by secondary coverage]; implied ~$4.1 per unit, consistent with the $4.95 launch price plus regional pricing. Lifetime to early Oct 2026: ≈ $26M–$38M (the $38M upper value is GameDiscoverCo's reported September figure, not re-verified) [ESTIMATE]. Spec method (8.5M × $5.99 ≈ $51M) overstates it because most copies sold at $4.95 or regional prices. Working figure for this study: ≥ $26M (floor), central ~$30M.</t>
         </is>
       </c>
       <c r="U13" s="3" t="inlineStr">
         <is>
-          <t>≈ $26M [ESTIMATE] = $38M gross − Steam cut (30% on first $10M = $3.0M; 25% on next $28M = $7.0M) = $28.0M × 0.93 (refunds/chargebacks) ≈ $26.0M to Dazed Games + Evil Landfall combined. The revenue split with Evil Landfall is undisclosed. Swedish corporate tax is not deducted.</t>
+          <t>≈ $18M–$26M [ESTIMATE]. At $26M gross: Steam cut 30% of first $10M ($3.0M) + 25% of $16M ($4.0M) = $7.0M → $19.0M × 0.93 ≈ $17.7M. At $38M gross: cut $3.0M + $7.0M = $10.0M → $28.0M × 0.93 ≈ $26.0M. Goes to Dazed Games + Evil Landfall combined (split undisclosed); Swedish corporate tax not deducted.</t>
         </is>
       </c>
       <c r="V13" s="3" t="inlineStr">
@@ -2862,12 +2862,12 @@
       </c>
       <c r="AF13" s="3" t="inlineStr">
         <is>
-          <t>(1) Publisher: the brief says self-published, and Steam lists Dazed Games as publisher, but CBR/TechTimes say it was 'published with support from' or 'bankrolled by' Evil Landfall. Chosen: self-published with Evil Landfall project investment and no equity. (2) All-time peak: 373,971 (SteamDB per GamesRadar/DLCompare, dated Aug 25 '5 days after launch' vs Aug 26) vs 373,887 (SteamCharts) vs 372,634 (Raijin). Chosen 373,971 on ~Aug 25–26. (3) Date of the 1M announcement: Aug 22 (most outlets) vs '3 days after launch' (TURGAME). Chosen Aug 22. (4) Reviews at 1M: 'nearly 12,000' (Techlomedia) vs ~13k (brief), so the implied ratio is a range of 77–83. (5) GameDiscoverCo: Aug gross $26M + Sep gross $6.5M = $32.5M, which does not reconcile with the stated '&gt;$38M LTD'. That could be a revision or different cut-off dates. Reported both and chose $38M as the latest. (6) Player count: the store says 1–4 players, while the wiki/patch notes say lobbies of up to 8 since 1.0.4. (7) Release plan: an April 2026 article said 'end of 2026' and the site said Q3 2026; the actual release was Aug 20. (8) Steam Page Analyzer's ~593k estimate is inconsistent with the confirmed 1M and was rejected.</t>
+          <t>(1) Publisher: the brief says self-published, and Steam lists Dazed Games as publisher, but CBR/TechTimes say it was 'published with support from' or 'bankrolled by' Evil Landfall. Chosen: self-published with Evil Landfall project investment and no equity. (2) All-time peak: 373,971 (SteamDB per GamesRadar/DLCompare, dated Aug 25 '5 days after launch' vs Aug 26) vs 373,887 (SteamCharts) vs 372,634 (Raijin). Chosen 373,971 on ~Aug 25–26. (3) Date of the 1M announcement: Aug 22 (most outlets) vs '3 days after launch' (TURGAME). Chosen Aug 22. (4) Reviews at 1M: 'nearly 12,000' (Techlomedia) vs ~13k (brief), so the implied ratio is a range of 77–83. (5) GameDiscoverCo: Aug gross $26M + Sep gross $6.5M = $32.5M, which does not reconcile with the stated '&gt;$38M LTD'. That could be a revision or different cut-off dates. Reported both and chose $38M as the latest. (6) Player count: the store says 1–4 players, while the wiki/patch notes say lobbies of up to 8 since 1.0.4. (7) Release plan: an April 2026 article said 'end of 2026' and the site said Q3 2026; the actual release was Aug 20. (8) Steam Page Analyzer's ~593k estimate is inconsistent with the confirmed 1M and was rejected. CROSS-CHECK 2026-10-08: GameDiscoverCo's August figures (6.3M+ units, ~$26M) were corroborated by secondary reports; the September '&gt;8.5M / &gt;$38M' figures could not be re-found, so the study uses the August readout as a floor and the September figures as an upper scenario.</t>
         </is>
       </c>
       <c r="AG13" s="3" t="inlineStr">
         <is>
-          <t>Post-launch: patches 1.0.4 (lobby limit 4→8), 1.0.5 (private invite-only lobbies), 1.0.12 on 2026-09-04 (Steam Cloud saves, last bug-fix-only patch), v1.1.0 'Islet Update' on 2026-09-28 (mini islands, Manta mini-boss, bow weapon, new bait/creatures/NPC/outfit/achievements, PEAK bundle), then 1.1.2/1.1.3 on 2026-09-29. Takeaways for a solo creator: (a) the first game failed commercially but taught the team marketing; (b) the publisher-light model (project investment, keep IP) can still bring a big label's halo; (c) months of weekly TikTok feature clips built the audience before launch; (d) a sub-$5 launch price plus co-op multi-pack buying produced roughly 80 units per review at the start, rising later. RELATED PRECEDENTS: WEBFISHING (Steam 2024-10-11, $4.99; developer and publisher 'lamedeveloper' (one person, per Steam listing); a remake of an 8-day 2022 itch.io game-jam project; cosy social fishing chatroom). Reviews: ~70,252, 97% positive (Raijin, 2026-07-22) / 69,258, ~97.5% (Vaporlens); just under 5,000 reviews, 98% positive, in launch week (Inverse). All-time peak CCU 23,838 (Tracker.gg). Sales are unconfirmed by the dev, and tracker estimates disagree widely: ~1.3M copies / ~$5.6M gross (Raijin, 2026-07-22, medium confidence); 1–2M owners (SteamSpy); ~5.06M / ~$25.2M (Vaporlens) [all ESTIMATE]. Engine (Godot) is unverified; it was not confirmed in this session's searches. Sources: https://raijin.gg/app/3146520/WEBFISHING , https://steamspy.com/dev/lamedeveloper , https://tracker.gg/population/steam/3146520 , https://www.inverse.com/gaming/steam-webfishing-cozy-chatroom-game-animal-crossing . It is the direct ancestor of the social-fishing hook, but How to Fish's peak CCU was ~16× higher. Fisch (Roblox, 2024) and Cast n Chill (2025, cosy idle fishing in a small desktop window): unverified, from memory only. Fisch shows fishing progression loops can scale to Roblox's young audience; Cast n Chill shows the 'desktop companion' idle-fishing niche. How to Fish combines the social fishing of WEBFISHING with PEAK-style physics-comedy co-op and shooter chaos.</t>
+          <t>Post-launch: patches 1.0.4 (lobby limit 4→8), 1.0.5 (private invite-only lobbies), 1.0.12 on 2026-09-04 (Steam Cloud saves, last bug-fix-only patch), v1.1.0 'Islet Update' on 2026-09-28 (mini islands, Manta mini-boss, bow weapon, new bait/creatures/NPC/outfit/achievements, PEAK bundle), then 1.1.2/1.1.3 on 2026-09-29. Takeaways for a solo creator: (a) the first game failed commercially but taught the team marketing; (b) the publisher-light model (project investment, keep IP) can still bring a big label's halo; (c) months of weekly TikTok feature clips built the audience before launch; (d) a sub-$5 launch price plus co-op multi-pack buying produced roughly 80 units per review at the start, rising later. RELATED PRECEDENTS: WEBFISHING (Steam 2024-10-11, $4.99; developer and publisher 'lamedeveloper' (one person, per Steam listing); a remake of an 8-day 2022 itch.io game-jam project; cosy social fishing chatroom). Reviews: ~70,252, 97% positive (Raijin, 2026-07-22) / 69,258, ~97.5% (Vaporlens); just under 5,000 reviews, 98% positive, in launch week (Inverse). All-time peak CCU 23,838 (Tracker.gg). Sales are unconfirmed by the dev, and tracker estimates disagree widely: ~1.3M copies / ~$5.6M gross (Raijin, 2026-07-22, medium confidence); 1–2M owners (SteamSpy); ~5.06M / ~$25.2M (Vaporlens) [all ESTIMATE]. Engine (Godot) is unverified; it was not confirmed in this session's searches. Sources: https://raijin.gg/app/3146520/WEBFISHING , https://steamspy.com/dev/lamedeveloper , https://tracker.gg/population/steam/3146520 , https://www.inverse.com/gaming/steam-webfishing-cozy-chatroom-game-animal-crossing . It is the direct ancestor of the social-fishing hook, but How to Fish's peak CCU was ~16× higher. Fisch (Roblox, 2024; not researched in this study) and Cast n Chill (2025, cosy idle fishing in a small desktop window; see B11 in this dataset). Fisch shows fishing progression loops can scale to Roblox's young audience; Cast n Chill shows the 'desktop companion' idle-fishing niche. How to Fish combines the social fishing of WEBFISHING with PEAK-style physics-comedy co-op and shooter chaos.</t>
         </is>
       </c>
       <c r="AH13" s="3" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>1 (solo developer) [CONFIRMED – developer's own Medium post written in first person; caller lead also describes Playrea as solo]</t>
+          <t>1 (solo developer) [CONFIRMED – developer's own Medium post written in first person]</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Soft launch Dec 2025 as 'Cannon Fest', renamed Smash Fest! in May 2026 (per caller lead – not independently re-verified; iOS app id 6748084174 suggests the store record dates from mid-2025)</t>
+          <t>Soft launch Dec 2025 as 'Cannon Fest', renamed Smash Fest! in May 2026 (per Diandian Data report – not independently re-verified; iOS app id 6748084174 suggests the store record dates from mid-2025)</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>no data – no source found giving Flow Games' headcount (7 searches across Gamigion, FoxData, mobilegamer.biz, LinkedIn/Crunchbase-type results). Founders are described as veterans of Peak Games (and, per caller lead, Good Job Games, Dream Games, Grand Games). Unverified whether the team is 5 or fewer; a studio of ex-Peak/Dream veterans shipping a polished live-ops hybrid-casual game is likely a small professional team (probably &gt;5 people), so do NOT treat it as a confirmed 1–5 person team.</t>
+          <t>no data – no source found giving Flow Games' headcount (7 searches across Gamigion, FoxData, mobilegamer.biz, LinkedIn/Crunchbase-type results). Founders are described as veterans of Peak Games (and, per a Diandian Data report, Good Job Games, Dream Games and Grand Games). Unverified whether the team is 5 or fewer; a studio of ex-Peak/Dream veterans shipping a polished live-ops hybrid-casual game is likely a small professional team (probably &gt;5 people), so do NOT treat it as a confirmed 1–5 person team.</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
@@ -6777,7 +6777,7 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>New studio; founders previously worked at Peak Games [ESTIMATE – Chinese trade report cited via FoxData/Baijing search results] and other Istanbul casual-game studios (Good Job Games, Dream Games, Grand Games per caller lead). The core mechanic is lifted from Peak's Toon Blast limited-time LiveOps event 'Cannon Fest' (cannonballs earned in match-3 levels used to clear objects in a separate event level), which explains both the soft-launch name and the later takedown.</t>
+          <t>New studio; founders previously worked at Peak Games [ESTIMATE – Chinese trade report cited via FoxData/Baijing search results] and other Istanbul casual-game studios (Good Job Games, Dream Games and Grand Games, per a Diandian Data report). The core mechanic is lifted from Peak's Toon Blast limited-time LiveOps event 'Cannon Fest' (cannonballs earned in match-3 levels used to clear objects in a separate event level), which explains both the soft-launch name and the later takedown.</t>
         </is>
       </c>
       <c r="L35" s="3" t="inlineStr">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="P35" s="3" t="inlineStr">
         <is>
-          <t>~2.9M downloads in the first month, 66.6% from the US [ESTIMATE – FoxData]; 6.41M iOS downloads in July 2026, #1 worldwide in iOS game downloads that month (up from #6) [ESTIMATE – FoxData]; 15M+ installs by end of July 2026 [ESTIMATE – AppMagic via Gamigion] vs 14.2M (another tracker) / 14.7M by August tally; August iOS ~5–6M (FoxData: down ~18% MoM; #2 iOS downloads behind Block Out!) [ESTIMATE]; run-rate ~300k downloads/day at peak [ESTIMATE – Gamigion analysis]. Cumulative by early Oct 2026: ~20–27M [ESTIMATE – 15M by end July + ~5–6M Aug + ~4–5M Sept assumed from declining trend; iOS-only after July]. US App Store ratings: ~232k (per caller lead, not re-verified).</t>
+          <t>~2.9M downloads in the first month, 66.6% from the US [ESTIMATE – FoxData]; 6.41M iOS downloads in July 2026, #1 worldwide in iOS game downloads that month (up from #6) [ESTIMATE – FoxData]; 15M+ installs by end of July 2026 [ESTIMATE – AppMagic via Gamigion] vs 14.2M (another tracker) / 14.7M by August tally; August iOS ~5–6M (FoxData: down ~18% MoM; #2 iOS downloads behind Block Out!) [ESTIMATE]; run-rate ~300k downloads/day at peak [ESTIMATE – Gamigion analysis]. Cumulative by early Oct 2026: ~20–27M [ESTIMATE – 15M by end July + ~5–6M Aug + ~4–5M Sept assumed from declining trend; iOS-only after July]. US App Store ratings: ~232k (AppFollow snapshot, Aug 2026; not re-verified).</t>
         </is>
       </c>
       <c r="Q35" s="3" t="inlineStr">
@@ -6937,7 +6937,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>In window (Next Fest demo June 2026, launch 2026-09-02). Placed in GROUP A, not B, because the team size could not be confirmed as ≤5 after 6 searches. The founder calls it a 'small independent team', but it is publisher-financed (TARK Games). Move to B if a headcount ≤5 is found.</t>
+          <t>In window (Next Fest demo June 2026, launch 2026-09-02). Placed in GROUP C (context case), not B, because the team size could not be confirmed as ≤5 after 6 searches. The founder calls it a 'small independent team', but it is publisher-financed (TARK Games).</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -7065,7 +7065,7 @@
       </c>
       <c r="AG36" s="3" t="inlineStr">
         <is>
-          <t>Group C = context case: team size could not be verified (described only as a 'small independent team' with publisher TARK financing), and the developer's 1M-copies claim conflicts with tracker estimates (~110k) and a very low review count (~3.5k). Kept for its Next Fest lesson. Group A because team size is unverified (see window_note). Lessons for a solo creator: (1) A one-line asymmetric co-op hook (each player has a different handicap) is extremely streamable and drives organic sharing. (2) A free Next Fest demo kept live after the fest can snowball: 6M demo players → 1M+ wishlists. (3) Paid conversion is much weaker than demo hype: 22.8k paid peak vs ~31k demo peak, and only ~3.5k reviews a month after launch despite 1M+ wishlists. This is consistent with the 0.10–0.15× wishlist-to-week-1 benchmark if units are ~110k–215k. (4) A publisher (TARK) supplied financing, creator relations and a Roblox adaptation; a solo developer would have to replace that with their own streamer outreach.</t>
+          <t>Group C = context case: team size could not be verified (described only as a 'small independent team' with publisher TARK financing), and the developer's 1M-copies claim conflicts with tracker estimates (~110k) and a very low review count (~3.5k). Kept for its Next Fest lesson.  Lessons for a solo creator: (1) A one-line asymmetric co-op hook (each player has a different handicap) is extremely streamable and drives organic sharing. (2) A free Next Fest demo kept live after the fest can snowball: 6M demo players → 1M+ wishlists. (3) Paid conversion is much weaker than demo hype: 22.8k paid peak vs ~31k demo peak, and only ~3.5k reviews a month after launch despite 1M+ wishlists. This is consistent with the 0.10–0.15× wishlist-to-week-1 benchmark if units are ~110k–215k. (4) A publisher (TARK) supplied financing, creator relations and a Roblox adaptation; a solo developer would have to replace that with their own streamer outreach.</t>
         </is>
       </c>
       <c r="AH36" s="3" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Built in a ~4-week jam; production cost &lt; $200k CONFIRMED.</t>
+          <t>Core built in a ~4-week jam; ~$200k production cost (reported, single secondary source).</t>
         </is>
       </c>
     </row>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>Built in ~9 weeks while the rest of the studio was on holiday; ~$54k est. cost.</t>
+          <t>Reportedly built by 4 devs in ~9 weeks while the rest of the studio was on holiday (single-source); ~$54k est. cost.</t>
         </is>
       </c>
     </row>
@@ -8048,26 +8048,26 @@
         <v>7.99</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>8.5</v>
+        <v>6.3</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>ESTIMATE (GameDiscoverCo, end Sep 2026); 1M CONFIRMED in 2 days</t>
+          <t>ESTIMATE floor (GameDiscoverCo Aug 2026, corroborated); up to ~8.5M by end Sep (unverified); 1M CONFIRMED in 2 days</t>
         </is>
       </c>
       <c r="J13" s="3" t="n">
         <v>374</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>ESTIMATE (GameDiscoverCo)</t>
+          <t>ESTIMATE floor (Aug 2026 only); up to ~$38M lifetime (unverified)</t>
         </is>
       </c>
       <c r="M13" s="3" t="n">
-        <v>26</v>
+        <v>17.7</v>
       </c>
       <c r="N13" s="3" t="n">
         <v>12</v>

</xml_diff>

<commit_message>
Add market report and finalize games analysis spreadsheet
report.md covers market trends, the How to Fish benchmark deep dive,
commonalities of viral small games, TOP 5 solo+AI opportunities with
2-4 week MVP plans, and a risk section with Steam/Roblox/web base rates.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W6mDjnjeBZpi9xGXrpYz1n
</commit_message>
<xml_diff>
--- a/game-market-research/games_analysis.xlsx
+++ b/game-market-research/games_analysis.xlsx
@@ -1149,7 +1149,7 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>~$200,000 total [ESTIMATE/reported – a single secondary (Italian-language) press report of the developers' figure; the 'under $200k' wording and the GDC 2026 talk ('Putting the Friends in Friendslop', Nick Kaman) could not be confirmed as the source in a cross-check on 2026-10-08]. Cross-check: 7 people × ~1–4 months × $6k ≈ $42k–170k [ESTIMATE].</t>
+          <t>&lt; $200,000 total [CONFIRMED – Game Developer: 'How co-op climbing hit Peak achieved 2 million sales for less than $200,000' (developer figures; see sources)]. Cross-check: 7 people × ~1–4 months × $6k ≈ $42k–170k [ESTIMATE].</t>
         </is>
       </c>
       <c r="W4" s="3" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="AF4" s="3" t="inlineStr">
         <is>
-          <t>Units: 10M+ (Aug 2025, Keighley/Alinea) and '11M on Steam' (GamesRadar 2026 headline) vs Raijin's ~7M (June 2026), which is clearly an underestimate; used 10–11M. The lead of 15.7M units / $87–92M could not be found in any source and was not used. '20M players' (June 2026, Aggro Crab) counts players, not purchases. Price: list $7.99 but launched at 38% off (~$4.95) and frequently discounted, so used Alinea's implied ~$5.67 realised price instead of 0.75 × list. Dev time: '4 weeks' (core jam) vs '~4 months' (total) – both reported. Peak CCU: 169,910–171k across trackers; used SteamDB-reported 170,759. CROSS-CHECK 2026-10-08: the production-cost figure was downgraded from CONFIRMED to reported/ESTIMATE because no English-language primary source was found.</t>
+          <t>Units: 10M+ (Aug 2025, Keighley/Alinea) and '11M on Steam' (GamesRadar 2026 headline) vs Raijin's ~7M (June 2026), which is clearly an underestimate; used 10–11M. The lead of 15.7M units / $87–92M could not be found in any source and was not used. '20M players' (June 2026, Aggro Crab) counts players, not purchases. Price: list $7.99 but launched at 38% off (~$4.95) and frequently discounted, so used Alinea's implied ~$5.67 realised price instead of 0.75 × list. Dev time: '4 weeks' (core jam) vs '~4 months' (total) – both reported. Peak CCU: 169,910–171k across trackers; used SteamDB-reported 170,759. CROSS-CHECK 2026-10-08: the '&lt; $200k' cost is supported by the Game Developer headline in the sources (and ~$200k by Italian press); a second independent search did not surface the article again.</t>
         </is>
       </c>
       <c r="AG4" s="3" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="W11" s="3" t="inlineStr">
         <is>
-          <t>~2–3 months: core fixed in ~1 week, then ~8 weeks to launch [reported – devs via Automaton/GamesIndustry.biz (Nordic Game 2026) and CEO Tim Badylak on LinkedIn ('launched just eight weeks after development began')]; Wikipedia/Icy Veins describe a summer-2025 game-jam project; press also says '3 months'. A cross-check search on 2026-10-08 could not re-find the interview, so treat '~9 weeks' as reported, not independently verified.</t>
+          <t>Just over 2 months (~9 weeks): core fixed in ~1 week, then ~8 weeks to launch [CONFIRMED – Automaton 2026-06-25 ('made as a breather in just over 2 months' by 4 devs, from a GamesIndustry.biz/Nordic Game 2026 interview); CEO Tim Badylak on LinkedIn: launched 'just eight weeks after development began']. Press also says '3 months' / 'summer 2025 game-jam project' (Icy Veins, Wikipedia).</t>
         </is>
       </c>
       <c r="X11" s="3" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="AF11" s="3" t="inlineStr">
         <is>
-          <t>Week-1 sales: 1.3M (dev CM, 2025-10-26/27) vs a report of '2.5M in first week' – the CEO's LinkedIn actually says 2.5M within two weeks; used that. A gamedev.net/GamesIndustry syndication said '2M units in eight days' – consistent with the trajectory. Dev time: '8 weeks' (CEO), '1 week + ~8 weeks' (Automaton), '3 months' (Icy Veins) – used ~9 weeks. Team: 4 devs built it (dev interview) vs 'five-person studio' (review) – 4 used for the game. Steam units now: Raijin 2.1M (contradicts confirmed 4.5M, discarded) vs Gamalytic 7.3M vs Boxleiter 5.3–7.1M – reported a range. Gross: Raijin $14M vs Gamalytic $45.4M vs own $27–36M. Xbox Game Pass date: Pure Xbox metadata May 2026 vs Xbox Wire 2026-06-30 – used Xbox Wire. Exact US price ($7.99 vs $8.99) not verified; GameDiscoverCo and Notebookcheck both say '$8' CROSS-CHECK 2026-10-08: the 4-developer / ~9-week build could not be re-found in an independent search; the 4.5M-by-December-2025 figure was corroborated by an aggregator (2.5–4.5M range).</t>
+          <t>Week-1 sales: 1.3M (dev CM, 2025-10-26/27) vs a report of '2.5M in first week' – the CEO's LinkedIn actually says 2.5M within two weeks; used that. A gamedev.net/GamesIndustry syndication said '2M units in eight days' – consistent with the trajectory. Dev time: '8 weeks' (CEO), '1 week + ~8 weeks' (Automaton), '3 months' (Icy Veins) – used ~9 weeks. Team: 4 devs built it (dev interview) vs 'five-person studio' (review) – 4 used for the game. Steam units now: Raijin 2.1M (contradicts confirmed 4.5M, discarded) vs Gamalytic 7.3M vs Boxleiter 5.3–7.1M – reported a range. Gross: Raijin $14M vs Gamalytic $45.4M vs own $27–36M. Xbox Game Pass date: Pure Xbox metadata May 2026 vs Xbox Wire 2026-06-30 – used Xbox Wire. Exact US price ($7.99 vs $8.99) not verified; GameDiscoverCo and Notebookcheck both say '$8' CROSS-CHECK 2026-10-08: the 4-developer / ~9-week build rests on the Automaton article in the sources (not re-found in a second search); the 4.5M-by-December-2025 figure was corroborated by an aggregator (2.5–4.5M range).</t>
         </is>
       </c>
       <c r="AG11" s="3" t="inlineStr">
@@ -7427,7 +7427,7 @@
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Core built in a ~4-week jam; ~$200k production cost (reported, single secondary source).</t>
+          <t>Core built in a ~4-week jam; production cost &lt; $200k (CONFIRMED via Game Developer).</t>
         </is>
       </c>
     </row>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>Reportedly built by 4 devs in ~9 weeks while the rest of the studio was on holiday (single-source); ~$54k est. cost.</t>
+          <t>Built by 4 devs in just over 2 months while the rest of the studio was on holiday (Automaton); ~$54k est. cost.</t>
         </is>
       </c>
     </row>

</xml_diff>